<commit_message>
Migrating VerifyFirst_Live_Product_Verification_104_Audit.xlsx to cloud
</commit_message>
<xml_diff>
--- a/VerifyFirst_Live_Product_Verification_104_Audit.xlsx
+++ b/VerifyFirst_Live_Product_Verification_104_Audit.xlsx
@@ -579,7 +579,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P105"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Foxtale Nourishing Moisturizer</t>
+          <t>Foxtale Nourishing Ceramide Moisturizer</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -1072,35 +1072,35 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>https://www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb?pid=MSCHN4UFYCHFCT4S</t>
+          <t>https://www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca?pid=MSCGNE2GYCJHYEBZ</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
+          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca%3Fpid%3DMSCGNE2GYCJHYEBZ</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
+          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca%3Fpid%3DMSCGNE2GYCJHYEBZ</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>Foxtale Brightening Moisturiser with Vitamin C &amp; Niacinamide|Brightens, Fades Dark Spots</t>
+          <t>Foxtale Nourishing Ceramide Moisturizer for Dry Skin, Skin-Barrier Repair &amp; Hydration (150 ml)</t>
         </is>
       </c>
       <c r="K7" s="15" t="n">
-        <v>279</v>
+        <v>484</v>
       </c>
       <c r="L7" s="15" t="n">
-        <v>345</v>
+        <v>747</v>
       </c>
       <c r="M7" s="15" t="n">
-        <v>66</v>
+        <v>263</v>
       </c>
       <c r="N7" s="16" t="n">
-        <v>19.1</v>
+        <v>35.2</v>
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Foxtale Nourishing Moisturizer</t>
+          <t>Foxtale Nourishing Ceramide Moisturizer</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1144,35 +1144,35 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb?pid=MSCHN4UFYCHFCT4S</t>
+          <t>https://www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca?pid=MSCH6GYQHDRR9CH4</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
+          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca%3Fpid%3DMSCH6GYQHDRR9CH4</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
+          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca%3Fpid%3DMSCH6GYQHDRR9CH4</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Foxtale Brightening Moisturiser with Vitamin C &amp; Niacinamide|Brightens, Fades Dark Spots</t>
+          <t>Foxtale Nourishing Ceramide Moisturizer for Dry Skin, Skin-Barrier Repair &amp; Hydration (100 ml)</t>
         </is>
       </c>
       <c r="K8" s="7" t="n">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>345</v>
+        <v>395</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>66</v>
+        <v>97</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>19.1</v>
+        <v>24.6</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Foxtale Nourishing Moisturizer</t>
+          <t>Foxtale Nourishing Ceramide Moisturizer</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -1216,35 +1216,35 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>https://www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb?pid=MSCHN4UFYCHFCT4S</t>
+          <t>https://www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca?pid=MSCGNF44HGHBPR8E</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
+          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca%3Fpid%3DMSCGNF44HGHBPR8E</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
+          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-nourishing-ceramide-moisturizer-dry-skin-skin-barrier-repair-hydration/p/itm54d45bb084cca%3Fpid%3DMSCGNF44HGHBPR8E</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>Foxtale Brightening Moisturiser with Vitamin C &amp; Niacinamide|Brightens, Fades Dark Spots</t>
+          <t>Foxtale Nourishing Ceramide Moisturizer for Dry Skin, Skin-Barrier Repair &amp; Hydration (50 ml)</t>
         </is>
       </c>
       <c r="K9" s="15" t="n">
-        <v>279</v>
+        <v>222</v>
       </c>
       <c r="L9" s="15" t="n">
-        <v>345</v>
+        <v>275</v>
       </c>
       <c r="M9" s="15" t="n">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="N9" s="16" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Foxtale Vit C Super Glow Moisturizer</t>
+          <t>Foxtale Brightening Moisturiser (Vit C &amp; Niacinamide)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1864,35 +1864,35 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>https://www.flipkart.com/foxtale-super-glow-moisturiser-4-vitc-niacinamide-complex-brighter-skin/p/itm90099ed5d84fb?pid=MSCGU7PUVYHD7UGA</t>
+          <t>https://www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb?pid=MSCHN4UFYCHFCT4S</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-super-glow-moisturiser-4-vitc-niacinamide-complex-brighter-skin/p/itm90099ed5d84fb%3Fpid%3DMSCGU7PUVYHD7UGA</t>
+          <t>https://verifyfirst.co.in/?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-super-glow-moisturiser-4-vitc-niacinamide-complex-brighter-skin/p/itm90099ed5d84fb%3Fpid%3DMSCGU7PUVYHD7UGA</t>
+          <t>https://alerts.zero483.com/deals.html?q=https%3A//www.flipkart.com/foxtale-brightening-moisturiser-vitamin-c-niacinamide-brightens-fades-dark-spots/p/itm897d92231c6cb%3Fpid%3DMSCHN4UFYCHFCT4S</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Foxtale Super Glow Moisturiser With 4% VitC-Niacinamide Complex For Brighter Skin</t>
+          <t>Foxtale Brightening Moisturiser with Vitamin C &amp; Niacinamide|Brightens, Fades Dark Spots (50 ml)</t>
         </is>
       </c>
       <c r="K18" s="7" t="n">
-        <v>401</v>
+        <v>279</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>495</v>
+        <v>345</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
@@ -8495,7 +8495,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:E30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -8637,8 +8637,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="B17" s="25" t="inlineStr">
         <is>

</xml_diff>